<commit_message>
Refresh Excel and CSVs with Douyin competitor merge
Merge task7 accounts/posts into root tables and 任务7 sheet after local Excel rebuild.
</commit_message>
<xml_diff>
--- a/research/jinan_tuoguan_2026/济南托管调研_v1.xlsx
+++ b/research/jinan_tuoguan_2026/济南托管调研_v1.xlsx
@@ -28,7 +28,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'任务4_企查查'!$A$1:$H$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'任务5_政府政策'!$A$1:$H$7</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'任务6_小红书'!$A$1:$E$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'任务7_抖音同城'!$A$1:$E$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'任务7_抖音同城'!$A$1:$E$133</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'任务8_场地租金'!$A$1:$F$18</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'任务9_人工成本'!$A$1:$E$17</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'任务10_学一家'!$A$1:$E$23</definedName>
@@ -11588,14 +11588,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
-    <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="10" customWidth="1" min="3" max="3"/>
-    <col width="10" customWidth="1" min="4" max="4"/>
-    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="34" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="100" customWidth="1" min="4" max="4"/>
+    <col width="72" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -11625,8 +11625,3572 @@
         </is>
       </c>
     </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>94年小王｜盘锦初中晚自习托管</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>卖点=实验中学新初一家长注意；爱顿校区安可托管中心环境展示；近30日估计=1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>万小妹</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>卖点=济南最美学校，绿城育华杨柳春风学校食堂；一蔬一饭藏教养；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>东街小学欣悦托辅</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>卖点=托管班大门已敞开，等待热爱学习的小小探索者 #开学季 #招生季；近30日估计=1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>乐思托辅</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>卖点=实验中学校区托管，只有12个床位，招满即可；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>乐恩托管</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>卖点=每一刻都值得被记录 #泉海学校 #乐恩托管 #晚辅日常；近30日估计=1</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>云朵中心</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>卖点=开学前一天校区安全、卫生标准讲解；近30日估计=1</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>六六托管中心闫老师🙋（高端，专业）</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>卖点=#托管 #济南；一心只做托管，用心用爱撑起托管的孩子！；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>努力的龙</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>卖点=谁家托管点100杯果汁啊 #托管班 #托管上班日常；近30日估计=1</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>十七小学繁星托管</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>卖点=开学两个星期了；做托管的是良心，尽心即可；近30日估计=1</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>博尔安亲托管中心官方号</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>卖点=专业托管用心让家长放心 #作业辅导 #课后服务；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>壹心托管济南校区</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 12 条</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>粉丝=1797；卖点=爱有温度，行有尺度；心存敬畏，事求极致。壹心托管胜利大街校区正式启航；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv；主页=https://www.douyin.com/user/MS4wLjABAAAAaUBMtA-9SvagxcGJfXlgx1eQ3S1oGfkTKxnmmtUJdH8MPRQLIdeQwSV6JfHrTsaO</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>大明湖的夏耦合</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>卖点=学校有配餐的建议二年级再去吃，小饭桌是刚需，但行业错综复杂。；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>天朗气清</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>卖点=#新学期 #托管 #一切为了孩子 #学习 #见证成长；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>天空教育官方号</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>账号；公开搜索结果账号</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>粉丝=855；卖点=济南市中区和槐荫区12年教培托管；午托、晚托、美术、书法；服务上万客户；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv；主页=https://www.douyin.com/user/MS4wLjABAAAAXB6u9Hfgy265b-Mn1mEsIIVncQ4_dyG7QwwDnkZFA4k8oZj5KjMFIr9tnef-3bwX</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>安馨托教｜西站路小学 52中午晚托</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>卖点=@安馨托教｜西站路小学 52中午晚托；近30日估计=1</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>小星星学堂【优优老师】</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>卖点=#实验中学 #实验托管 #托管日常；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>开托管的80后</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>卖点=托管招生 #托管；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>彩虹泡泡教育管家</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>卖点=济南儿童成长陪伴师 #济南 #儿童成长陪伴 #女性创业；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>悦维美刻托管济南站</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>卖点=像这样的品牌托管今年就会开在济南各个中学门口 #中学生托管中心 #济南中学生托管；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>成立志</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>卖点=志立成长中心开始招生；自理、自立，做真教育；近30日估计=1</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>新智托管</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>卖点=托管老师日常：接娃、维持秩序、订正错题，沉浸式辅导；近30日估计=1</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>李星野</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>卖点=用心、长久、安全；靠实打实的口碑积累记录托管校区成长；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>泉海托管</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>卖点=济南泉海学校附近专业托辅 #托管 #泉海学校 #素养课堂；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>济南书墨托管李老师</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>账号；公开搜索结果账号</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>粉丝=3741；卖点=20年儿童教育；中小学精品托管；辅导过济南中小学生；有温度的托管班；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv；主页=https://www.douyin.com/user/MS4wLjABAAAA-XE1-eX-ShMbHMdNFxFd9rBmyxb8UFySlyvYsFcyC7Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>济南书法飒老师</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>卖点=开学第一天 #新学期托管 #缘承托管 #专业晚辅 #济南托管 #西客站；近30日估计=1</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>济南卓安官方号</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>卖点=#济南托管 #小班托管 #济南同城 #卓安 #课后陪伴；近30日估计=1</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>济南卓阳优托</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>账号；公开搜索结果账号</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>粉丝=1306；卖点=天桥区老牌托管；专业师资；暖心托管；靠谱托管让家长安心；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv；主页=https://www.douyin.com/user/MS4wLjABAAAASnqzITf1VyCBa2Zt-mgaoo74JTZhRMAiU4ZJRv3aLisQNv22w9uf_T6HpiZuL1BM</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>济南天才自助餐托管中心</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>卖点=把饭做好，孩子吃饱，家长认可，这就是口碑 #托管用餐 #学生餐；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>济南学成课后中心</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>账号；公开搜索结果账号</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>粉丝=1109；卖点=在济南开托管10年的老托管人；两家校区，经五路+万科城；欢迎参观咨询；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv；主页=https://www.douyin.com/user/MS4wLjABAAAApCAPQqLg4mwNCO4t_btg-aiUQrs7ioXegGPVB0vyZ5o</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>济南市快乐助学坊成长中心～李老师</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 2 条</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>卖点=济南家长圈有口皆碑！19年0投诉托管班；接娃+辅导+晚餐全包 #济南托管 #快乐助学坊；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>济南市槐荫区惠心托管中心</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>粉丝=451；卖点=幼儿园园长转型；多年幼教管理；懂教育、懂孩子、重安全；800㎡空间；近30日估计=1</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv；主页=https://www.douyin.com/user/MS4wLjABAAAAWdUDcQpSeHIiHy_bMc9BwZSfsRjrQaxuhgvih2V3S4Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>济南慧学优安托</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>账号；公开搜索结果账号</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>粉丝=2135；卖点=高端托管；15年教育旅程；教育理念与托管日常；梦想乐园；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv；主页=https://www.douyin.com/user/MS4wLjABAAAAM2VEn5oqax3vnF-X5IwPw3smJq6p-MZ-o4l85pRh4Pp8cWyB9FDqPynHIeJtIwyI</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>济南托管王校长</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>账号；公开搜索结果账号</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>粉丝=1854；卖点=教育从业20年；专业晚辅、培优、午餐午休；从小托管做成百人大校；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv；主页=https://www.douyin.com/user/MS4wLjABAAAAVt6NUO0w1inbThSBgrXFgWmgQNMAMm2EDy2CASLfO-E</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>济南托管郑老师</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>卖点=#济南 #济南托管 #济南托管郑老师 #济南托管哪家好？ 来看看投资400万托管的秘密吧；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>济南托管高老师</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>账号；公开搜索结果账号</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>粉丝=2096；卖点=十几年经验；小学生午托、晚托；习惯培养，不只接送、吃饭、写作业；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv；主页=https://www.douyin.com/user/MS4wLjABAAAAIYA9gydLiokUYk3crHxZ2YAhhh7ewb0WkYC23gR4gZo</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>济南无忧托管</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>账号；公开搜索结果账号</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>粉丝=152；卖点=托您所爱、管您所忧；胜利大街小学托管；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv；主页=https://www.douyin.com/user/MS4wLjABAAAAvmz3VbMJzu2DRKl8OecxleSbqSjlnDL1AHdLw67dLxM</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>济南杨柳春风（正信置业）</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 2 条</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>卖点=#小春风播报 #名校；学校师资水平介绍；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>济南槐荫123托管成长中心</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>账号；公开搜索结果账号</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>粉丝=0；卖点=8年小学托管；作业辅导、安全接送、营养晚餐、书法/阅读作文/英语启蒙；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv；主页=https://www.douyin.com/user/MS4wLjABAAAAVEn7Mb8t2LbYbQ2XMsDXYbOtVqM6uIGEdX1hTCzzeZ9sF3SCZYh8-XTVlkdeKTU3</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>济南槐荫小火竹官方号</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 4 条</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>粉丝=350；卖点=00后美院本科生，四年托管经验，23岁孤注一掷，耗资百万打造槐荫托管天花板！#高端托管中心 #小学生托管 #作业辅导托管；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv；主页=https://www.douyin.com/user/MS4wLjABAAAAH3zONTSzG-Yo8-aLh505CHGPCjQ44e6T_8Q8vtbdbHffbHdReSXOvN7aCEXuBK</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>济南槐荫顺馨教育</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>账号；公开搜索结果账号</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>粉丝=477；卖点=午餐午休、晚托作业、习惯养成、周末/假期托管；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv；主页=https://www.douyin.com/user/MS4wLjABAAAAlHNe8n-9xHljuFjafYgSaoFNlWudMuYbIYEXVVCPHMs</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>济南老董</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>卖点=上小学了要不要报小饭桌？家长经验分享 #济南小学 #济南小饭桌；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>济南蜗牛等等托育服务有限公司</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>账号；公开搜索结果账号</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>粉丝=2117；卖点=济南托育示范点；自然教育；招生0-4岁；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv；主页=https://www.douyin.com/user/MS4wLjABAAAAx9hspCfPAWOr_cphRDSG9euBmHM_IAgEr8iabDWpv7AbgwPHaeSuQdx_GjNhyMXa</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>省实验校内王老师</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 2 条</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>卖点=开学了！#济南 #小饭桌 #日常 #vlog；近30日估计=2</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>章丘托管金八力刘笑</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>卖点=退让换来的是无底线的伤害，这次我一定刚到底！#章丘托管 #章丘托管班；近30日估计=1</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>精心托管槐荫区医学中心小学宸园北区12号</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 2 条</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>卖点=精心托管新校区已规整完毕，地址：宸园北区12-2-101，静候小朋友归来；近30日估计=2</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>美吉精品托管</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>卖点=七里河区西站美吉精品托管火热招生中；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>老谢家的二姑娘</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>卖点=一日托管流程，期待更多的宝贝加入我们 #托管；近30日估计=1</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>花锦时代</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>粉丝=1；卖点=槐荫实验学校附近晚辅：20人以下小班、作业全查、错题精讲、接送方便、健康晚餐；原价880元/月，前10名首月减100元，39.9元体验3天含晚餐；公开价格=880元/月；近30日估计=1</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv；主页=https://www.douyin.com/user/MS4wLjABAAAAPJ3lf0Jz5HvHFxnqgUtQkrwjiIGy7VyZ8DqxCHK6gjeHBgWjC_IgmDr3PMkR1Qzq</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>萌雅童乐托管</t>
+        </is>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>粉丝=234；卖点=原槐荫区营市街幼儿园；普惠、传统文化、鼓乐、书法、棋类等；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv；主页=https://www.douyin.com/user/MS4wLjABAAAAGhzQAX8Wg_JxYiCpwrDq2J01qUtQjHFgtCQtHAh5TpPfZGu35AL3KWgCMKZSkiwG</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>营东小学天天托管来啦</t>
+        </is>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 2 条</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>卖点=#新学期新开始 #托管 招生啦；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>诺德城依春然托管</t>
+        </is>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>卖点=关于依春然；托管班、小饭桌、小学；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>贝尔优能任兴校区</t>
+        </is>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>卖点=实验学校附近报托管就找王老师；专业、更靠谱；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>贝尔安亲课后托管加盟</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>卖点=实地探访，学期收费17800元的托管；托管收费与餐食探店；公开价格=17800元；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>郑老师教育</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>账号；公开搜索结果账号</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>粉丝=6191；卖点=30+分校；分享幼升小、小升初、中高考择校规划、政策解读、真题干货；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv；主页=https://www.douyin.com/user/MS4wLjABAAAAdArEeYtGLBCQbbkSqrb0f3Y1yA9oXFc9VNsxCSjRzYynuKGtkqvsk8zauvz-fK8S</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>长清恒大育贤博跃托管—李老师</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>卖点=好的习惯在日复一日的陪伴中悄然生根；近30日估计=1</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>长清黑美人</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>卖点=长清一家做的非常好的托管，济南的都过来学习交流！#托管 #长清托管；近30日估计=1</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>静慧托管～雪婷</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>卖点=晚辅但不是普通晚辅；标准化流程、个性化一对一辅导；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>龙兴之家 课后伴学</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>粉丝=18；卖点=泉景小学对门托管；每日新鲜食材，荤素均衡搭配；龙兴之家课后伴学；近30日估计=1</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv；主页=https://www.douyin.com/user/MS4wLjABAAAAE5vr1pF_dwIVY_z7c8rmU50N5jVwmhyfXn50od8SM4i2PFlOFNZMLNWF8vAfXGFd</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>龚老师和她的托管朋友</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>卖点=和托管老师闹过别扭，换了几家对比后觉得这家靠谱；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>ꕥ多财💞多亿</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 2 条</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>卖点=泉景小学附近新开托管，做接校、托管、寒暑假、餐食和作业反馈 #泉景小学 #卧龙花园；近30日估计=0</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>🌈俊霖托管🌈</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>卖点=关于秋季晚辅，随便问 #秋季晚辅 #小学 #初中；近30日估计=1</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>💕济南武老师教育精品一站式托辅✨</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>账号；公开主页；采样帖子 1 条</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>卖点=#营市东街 做一家让家长认可省心的托管机构；近30日估计=1</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/accounts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>帖子｜济南托管郑老师</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>帖子；2025年1月17日</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>赞=42；时长=01:32；#济南 #济南托管 #济南托管郑老师 #济南托管哪家好？ 来看看投资400万托管的秘密吧</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>帖子｜济南市快乐助学坊成长中心～李老师</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>帖子；2025年3月20日</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>赞=93；时长=01:41；济南家长圈有口皆碑！19年0投诉托管班；接娃+辅导+晚餐全包 #济南托管 #快乐助学坊</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>帖子｜壹心托管济南校区</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>帖子；6月29日</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>赞=10；时长=00:50；爱有温度，行有尺度；心存敬畏，事求极致。壹心托管胜利大街校区正式启航</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>帖子｜章丘托管金八力刘笑</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>帖子；8月25日</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>赞=456；时长=02:26；退让换来的是无底线的伤害，这次我一定刚到底！#章丘托管 #章丘托管班</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>帖子｜济南槐荫小火竹官方号</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>帖子；5月13日</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>赞=98；时长=00:54；00后美院本科生，四年托管经验，23岁孤注一掷，耗资百万打造槐荫托管天花板！#高端托管中心 #小学生托管 #作业辅导托管</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>帖子｜长清黑美人</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>帖子；8月30日</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>赞=240；时长=03:31；长清一家做的非常好的托管，济南的都过来学习交流！#托管 #长清托管</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>帖子｜省实验校内王老师</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>帖子；8月22日</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>赞=39；时长=01:28；开学了！#济南 #小饭桌 #日常 #vlog</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>帖子｜彩虹泡泡教育管家</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>帖子；2025年3月13日</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>赞=48；时长=02:31；济南儿童成长陪伴师 #济南 #儿童成长陪伴 #女性创业</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>帖子｜悦维美刻托管济南站</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>帖子；2025年5月2日</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>赞=20；时长=00:54；像这样的品牌托管今年就会开在济南各个中学门口 #中学生托管中心 #济南中学生托管</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>帖子｜济南槐荫小火竹官方号</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>帖子；5月13日</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>赞=98；时长=00:54；00后美院本科生，四年托管经验，耗资百万打造槐荫托管天花板！#高端托管中心 #小学生托管 #作业辅导托管</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>帖子｜🌈俊霖托管🌈</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>帖子；8月20日</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>赞=2；时长=00:29；关于秋季晚辅，随便问 #秋季晚辅 #小学 #初中</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>帖子｜济南市槐荫区惠心托管中心</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>帖子；13小时前</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>赞=6；时长=00:55；一晃十五年过去了，这段时光里有收获，也有遗憾。</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>帖子｜开托管的80后</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>帖子；3月4日</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>赞=8；时长=图文；托管招生 #托管</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>帖子｜精心托管槐荫区医学中心小学宸园北区12号</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>帖子；8月27日</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>赞=2；时长=图文；精心托管新校区已规整完毕，地址：宸园北区12-2-101，静候小朋友归来</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>帖子｜精心托管槐荫区医学中心小学宸园北区12号</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>帖子；6天前</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>赞=6；时长=图文；教师节到了，送给一线老师们，细心用心教育陪伴孩子</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>帖子｜济南卓安官方号</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>帖子；1天前</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>赞=9；时长=00:32；#济南托管 #小班托管 #济南同城 #卓安 #课后陪伴</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>帖子｜济南槐荫小火竹官方号</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>帖子；7月28日</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>赞=18；时长=00:33；高投入的托管中心，哪里区别于普通小饭桌？#槐荫区托管 #小火竹托管</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>帖子｜大明湖的夏耦合</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>帖子；2021年5月30日</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>赞=1164；时长=01:06；学校有配餐的建议二年级再去吃，小饭桌是刚需，但行业错综复杂。</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>帖子｜省实验校内王老师</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>帖子；7月25日</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>赞=38；时长=01:25；沉浸式体验高中小饭桌做饭的一天 #日常 #vlog #济南</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>帖子｜壹心托管济南校区</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>帖子；2025年9月15日</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>赞=22；时长=00:18；百万级别小饭桌，都给孩子们吃什么？带大家看一看</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>帖子｜壹心托管济南校区</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>帖子；2025年11月23日</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>赞=166；时长=00:16；与根posts.csv post_id=7575856001335147953匹配，未重复追加；托管天花板，神仙小饭桌，就是这么硬核 #济南壹心托管</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>帖子｜济南老董</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>帖子；6月18日</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>赞=33；时长=03:00；上小学了要不要报小饭桌？家长经验分享 #济南小学 #济南小饭桌</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>帖子｜济南天才自助餐托管中心</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>帖子；6月3日</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>赞=14；时长=02:16；把饭做好，孩子吃饱，家长认可，这就是口碑 #托管用餐 #学生餐</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>帖子｜天朗气清</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>帖子；2025年8月22日</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>赞=4；时长=01:28；#新学期 #托管 #一切为了孩子 #学习 #见证成长</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>帖子｜ꕥ多财💞多亿</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>帖子；6月23日</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>赞=5；时长=图文；泉景小学附近新开托管，做接校、托管、寒暑假、餐食和作业反馈 #泉景小学 #卧龙花园</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>帖子｜龙兴之家 课后伴学</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>帖子；3天前</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>赞=9；时长=图文；泉景小学对门托管；每日新鲜食材，荤素均衡搭配；龙兴之家课后伴学</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>帖子｜ꕥ多财💞多亿</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>帖子；6月18日</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>赞=5；时长=00:20；泉景中学对面19号楼托管开业，幼小衔接，一二年级 #卧龙花园 #泉景中学</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>帖子｜济南市快乐助学坊成长中心～李老师</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>帖子；2025年3月20日</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>赞=93；时长=01:41；济南家长圈有口皆碑！19年0投诉；接娃+辅导+晚餐全包</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>帖子｜壹心托管济南校区</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>帖子；2025年7月26日</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>赞=15；时长=00:32；托管天花板，神仙小饭桌，吃货娃挑食娃都来做壹心的娃 #泉海学校</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>帖子｜努力的龙</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>帖子；8月5日</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>赞=102；时长=01:14；谁家托管点100杯果汁啊 #托管班 #托管上班日常</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>帖子｜济南书法飒老师</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>帖子；9月1日</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>赞=10；时长=00:12；开学第一天 #新学期托管 #缘承托管 #专业晚辅 #济南托管 #西客站</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>帖子｜六六托管中心闫老师🙋（高端，专业）</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>帖子；3月7日</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>赞=17；时长=03:39；#托管 #济南；一心只做托管，用心用爱撑起托管的孩子！</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>帖子｜安馨托教｜西站路小学 52中午晚托</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>帖子；8月21日</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>赞=14；时长=00:09；@安馨托教｜西站路小学 52中午晚托</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>帖子｜美吉精品托管</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>帖子；2025年8月22日</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>赞=17；时长=01:01；七里河区西站美吉精品托管火热招生中</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>帖子｜贝尔安亲课后托管加盟</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>帖子；3月20日</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>赞=251；时长=03:45；公开价格=17800元；实地探访，学期收费17800元的托管；托管收费与餐食探店</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>帖子｜💕济南武老师教育精品一站式托辅✨</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>帖子；8月29日</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>赞=11；时长=00:23；#营市东街 做一家让家长认可省心的托管机构</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>帖子｜营东小学天天托管来啦</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>帖子；2024年8月30日</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>赞=5；时长=00:30；#新学期新开始 #托管 招生啦</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>帖子｜萌雅童乐托管</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>帖子；2022年8月2日</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>赞=26；时长=02:44；营市街幼儿园位于营市东街44号；普惠性幼儿园，传统文化、鼓乐、书法、棋类等特色课程</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>帖子｜李星野</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>帖子；7月23日</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>赞=149；时长=00:59；用心、长久、安全；靠实打实的口碑积累记录托管校区成长</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>帖子｜老谢家的二姑娘</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>帖子；8月23日</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>赞=36；时长=01:20；一日托管流程，期待更多的宝贝加入我们 #托管</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>帖子｜东街小学欣悦托辅</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>帖子；8月31日</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>赞=27；时长=02:43；托管班大门已敞开，等待热爱学习的小小探索者 #开学季 #招生季</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>帖子｜营东小学天天托管来啦</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>帖子；2024年7月10日</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>赞=4；时长=00:15；下午数学课学习；理论与实践结合 #营市东街小学 #天天托管</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>帖子｜花锦时代</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>帖子；8月22日</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>赞=0；时长=图文；公开价格=880元/月；槐荫实验学校附近晚辅：20人以下小班、作业全查、错题精讲、接送方便、健康晚餐；原价880元/月，前10名首月减100元，39.9元体验3天含晚餐</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>帖子｜贝尔优能任兴校区</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>帖子；3月20日</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>赞=50；时长=00:33；实验学校附近报托管就找王老师；专业、更靠谱</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>帖子｜小星星学堂【优优老师】</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>帖子；4月22日</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>赞=11；时长=00:22；#实验中学 #实验托管 #托管日常</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>帖子｜壹心托管济南校区</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>帖子；2025年6月26日</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>赞=37；时长=03:19；与根posts.csv post_id=7520469530099993914匹配，未重复追加；校区从市场调研到落地成型；记录建设过程 #高端托管 #泉海中学</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>帖子｜济南槐荫小火竹官方号</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>帖子；7月28日</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>赞=6；时长=00:53；高投入的托管中心，哪里区别于普通小饭桌？</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>帖子｜万小妹</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>帖子；5月18日</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>赞=61；时长=02:56；济南最美学校，绿城育华杨柳春风学校食堂；一蔬一饭藏教养</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>帖子｜济南杨柳春风（正信置业）</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>帖子；2021年11月1日</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>赞=344；时长=01:27；#小春风播报 #名校；学校师资水平介绍</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>帖子｜龚老师和她的托管朋友</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>帖子；6月16日</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>赞=286；时长=00:08；和托管老师闹过别扭，换了几家对比后觉得这家靠谱</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>帖子｜十七小学繁星托管</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>帖子；2天前</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>赞=14；时长=00:31；开学两个星期了；做托管的是良心，尽心即可</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>帖子｜诺德城依春然托管</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>帖子；2025年8月16日</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>时长=关于依春然；关于依春然；托管班、小饭桌、小学</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>帖子｜济南杨柳春风（正信置业）</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>帖子；2022年3月1日</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>赞=105；时长=05:46；绿城育华杨柳春风幼儿园云参观 #济南</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>帖子｜长清恒大育贤博跃托管—李老师</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>帖子；16小时前</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>赞=6；时长=01:49；好的习惯在日复一日的陪伴中悄然生根</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>帖子｜壹心托管济南校区</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>帖子；2025年8月21日</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>赞=25；时长=02:04；什么情况啊来了就不想走的托管见过么 #济南壹心托管</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>帖子｜壹心托管济南校区</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>帖子；2025年7月5日</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>赞=7；时长=01:39；市中区泉海学校对面开了一家星级托管，出校门步行一分钟</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>帖子｜壹心托管济南校区</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>帖子；2025年7月24日</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>赞=13；时长=00:36；做托管要站在家长角度，用真心换放心</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>帖子｜新智托管</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>帖子；1天前</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>赞=23；时长=04:57；托管老师日常：接娃、维持秩序、订正错题，沉浸式辅导</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>帖子｜静慧托管～雪婷</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>帖子；6月24日</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>时长=晚辅标准化；晚辅但不是普通晚辅；标准化流程、个性化一对一辅导</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>帖子｜成立志</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>帖子；8月23日</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>赞=49；时长=00:38；志立成长中心开始招生；自理、自立，做真教育</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>帖子｜乐思托辅</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>帖子；7月3日</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>赞=6；时长=00:32；实验中学校区托管，只有12个床位，招满即可</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>帖子｜壹心托管济南校区</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>帖子；2025年7月11日</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>赞=48；时长=00:42；与根posts.csv post_id=7525763465560313146匹配，未重复追加；壹心只做一件事，用心做好一件事；托管正式启航</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>帖子｜94年小王｜盘锦初中晚自习托管</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>帖子；8月14日</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>赞=3；时长=01:16；实验中学新初一家长注意；爱顿校区安可托管中心环境展示</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>帖子｜云朵中心</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>帖子；8月31日</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>赞=83；时长=04:37；开学前一天校区安全、卫生标准讲解</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>帖子｜博尔安亲托管中心官方号</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>帖子；2023年4月8日</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>赞=8；时长=02:35；专业托管用心让家长放心 #作业辅导 #课后服务</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>帖子｜壹心托管济南校区</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>帖子；2025年10月14日</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>赞=19；时长=00:33；上学的孩子拼脑力也是拼体力，为泉海校区娃娃成长助力，用心做好每一餐</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>帖子｜壹心托管济南校区</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>帖子；2025年12月20日</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>赞=15；时长=00:29；这里是济南壹心托管泉海校区；很高兴认识你</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>帖子｜泉海托管</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>帖子；3月21日</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>赞=3；时长=00:29；济南泉海学校附近专业托辅 #托管 #泉海学校 #素养课堂</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>帖子｜乐恩托管</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>帖子；5小时前</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>赞=0；时长=00:17；每一刻都值得被记录 #泉海学校 #乐恩托管 #晚辅日常</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>帖子｜壹心托管济南校区</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>douyin</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>帖子；2025年8月5日</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
+        <is>
+          <t>赞=12；时长=00:28；想要了解的过来看看吧 #每日分享</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>02_douyin_competitors/posts.csv</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E1"/>
+  <autoFilter ref="A1:E133"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>